<commit_message>
Add Params & Benchmarks tab for Nemotron, Fable, Sol, Kimi K3, GLM, Qwen, DeepSeek
- New workbook sheet with total/active parameters, architecture, AA
  Intelligence Index, cost per task, GPQA Diamond, SWE-bench Verified/Pro,
  Terminal-Bench, HLE, pricing, and weekly token volume for 9 models
- CSV export data/csv/params_benchmarks.csv
- Documented sourcing and comparability caveats in data/README.md

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Model Comparison" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Top 20 Volume Chart" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By Developer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Params &amp; Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
@@ -22,12 +23,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.000"/>
     <numFmt numFmtId="167" formatCode="$#,##0.0"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="$0.00"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -112,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +149,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -373,6 +381,112 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>GPQA Diamond vs AA Intelligence Index</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Params &amp; Benchmarks'!H5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Params &amp; Benchmarks'!$A$6:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Params &amp; Benchmarks'!$H$6:$H$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Params &amp; Benchmarks'!J5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Params &amp; Benchmarks'!$A$6:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Params &amp; Benchmarks'!$J$6:$J$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -410,6 +524,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -20221,4 +20362,881 @@
   <autoFilter ref="A1:F49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter and benchmark deep-dive: selected model families</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron, Claude Fable, OpenAI GPT-5.6 Sol, Kimi K3, Z.ai GLM, Qwen, DeepSeek - researched 2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark scores are vendor-reported (highest reasoning effort) unless noted; harnesses differ across labs, so treat cross-model comparisons as approximate. AA = Artificial Analysis Intelligence Index v4.1 leaderboard snapshot, 2026-07-20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Total params (B)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Active params (B)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Architecture / license</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>AA Intelligence Index</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>AA cost per task ($)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>GPQA Diamond (%)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>SWE-bench Verified (%)</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>SWE-bench Pro (%)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Terminal-Bench (%)</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>TB ver.</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>HLE (%)</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Input $/1M</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Output $/1M</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Weekly tokens (B)</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Notes / sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 Ultra</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>550</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid Mamba-Transformer MoE (90% sparsity)</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>38</v>
+      </c>
+      <c r="I6" s="31" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J6" s="32" t="n">
+        <v>87</v>
+      </c>
+      <c r="K6" s="32" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="L6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="32" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="O6" s="32" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="P6" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Q6" s="20" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="R6" s="25" t="n">
+        <v>3316.038765601</v>
+      </c>
+      <c r="S6" s="33" t="inlineStr">
+        <is>
+          <t>Largest US open-weights model; NVIDIA model card (BF16). AA scored it 47.7-48.2 on Index v4.0 at release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 Super</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>120</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid Mamba-Transformer LatentMoE, NVFP4 pretraining</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" s="31" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="J7" s="32" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="K7" s="32" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M7" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O7" s="32" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="P7" s="20" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="Q7" s="20" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="R7" s="25" t="n">
+        <v>284.860456781</v>
+      </c>
+      <c r="S7" s="33" t="inlineStr">
+        <is>
+          <t>SWE-bench Verified via OpenHands harness (NVIDIA model card).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Undisclosed (Mythos-class; third-party estimates ~3T)</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" s="31" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J8" s="32" t="n">
+        <v>92.59999999999999</v>
+      </c>
+      <c r="K8" s="32" t="n">
+        <v>95</v>
+      </c>
+      <c r="L8" s="32" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="M8" s="32" t="n">
+        <v>88</v>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="O8" s="32" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="P8" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="R8" s="25" t="n">
+        <v>375.285408732</v>
+      </c>
+      <c r="S8" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic launch materials / system card; OpenAI's comparison table reports Terminal-Bench 83.1 and SWE-bench Pro 80.0. AA config: Adaptive Reasoning, Max Effort, Opus 4.8 fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Undisclosed (third-party estimates ~3T)</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>59</v>
+      </c>
+      <c r="I9" s="31" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J9" s="32" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="32" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="M9" s="32" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="O9" s="32" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="R9" s="25" t="n">
+        <v>411.249519808</v>
+      </c>
+      <c r="S9" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI launch table (Codex harness); no SWE-bench Verified published. AA config: max reasoning effort. HLE is AA-HLE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Stable LatentMoE, 16/896 experts active; KDA attention (active params ~50B, third-party estimate)</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>57</v>
+      </c>
+      <c r="I10" s="31" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J10" s="32" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="32" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="O10" s="32" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="P10" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="R10" s="25" t="n">
+        <v>12.051888516</v>
+      </c>
+      <c r="S10" s="33" t="inlineStr">
+        <is>
+          <t>First open 3T-class model; weights promised by 2026-07-27. Moonshot tech blog (reasoning_effort max, KimiCode harness); no SWE-bench results published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>753</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>MoE, MIT license; trained on Huawei Ascend 910B</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>51</v>
+      </c>
+      <c r="I11" s="31" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J11" s="32" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="K11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L11" s="32" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="M11" s="32" t="n">
+        <v>81</v>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="O11" s="32" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="P11" s="20" t="n">
+        <v>0.9366</v>
+      </c>
+      <c r="Q11" s="20" t="n">
+        <v>2.9436</v>
+      </c>
+      <c r="R11" s="25" t="n">
+        <v>3515.340760024</v>
+      </c>
+      <c r="S11" s="33" t="inlineStr">
+        <is>
+          <t>Z.ai release blog (Terminus-2 harness); strongest open-weights model on the AA Index. No SWE-bench Verified published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>Undisclosed (API-only; Qwen's top tier is closed since late 2025)</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>46</v>
+      </c>
+      <c r="I12" s="31" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J12" s="32" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="K12" s="32" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="L12" s="32" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="M12" s="32" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="N12" s="19" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O12" s="32" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P12" s="20" t="n">
+        <v>1.475</v>
+      </c>
+      <c r="Q12" s="20" t="n">
+        <v>4.425</v>
+      </c>
+      <c r="R12" s="25" t="n">
+        <v>162.911604779</v>
+      </c>
+      <c r="S12" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba Qwen3.7 release blog (xhigh reasoning).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>49</v>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>MoE with hybrid CSA+HCA attention, MIT license</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="I13" s="31" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J13" s="32" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="K13" s="32" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="L13" s="32" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="M13" s="32" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="N13" s="19" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O13" s="32" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="P13" s="20" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="Q13" s="20" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="R13" s="25" t="n">
+        <v>2473.441480536</v>
+      </c>
+      <c r="S13" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 technical report, Think-Max mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>284</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>MoE with hybrid CSA+HCA attention, MIT license</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="I14" s="31" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J14" s="32" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="K14" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="L14" s="32" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="M14" s="32" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="N14" s="19" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="O14" s="32" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="P14" s="20" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="Q14" s="20" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="R14" s="25" t="n">
+        <v>5240.398974088</v>
+      </c>
+      <c r="S14" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 technical report, Think-Max mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Total/active parameters: official vendor disclosures for open-weights models. Anthropic, OpenAI, and Alibaba do not disclose parameter counts for Fable 5, GPT-5.6 Sol, or Qwen3.7 Max; ~3T figures are third-party estimates only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Kimi K3's ~50B active is a community estimate from the disclosed 16-of-896 expert activation; Moonshot has not published an official active-parameter figure. Weights promised by 2026-07-27 (API-only as of 2026-07-20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Terminal-Bench versions differ (2.0 vs 2.1) and each lab uses its own agent harness (KimiCode, Claude Code, Codex, Terminus-2), so scores are not strictly comparable across rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>SWE-bench Pro validity is contested: OpenAI's 2026-07-08 audit estimates ~30% of tasks are flawed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>AA cost per task = Artificial Analysis's measured cost to run its Intelligence Index suite, divided per task; reflects token efficiency as well as list price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>HLE = Humanity's Last Exam, no tools (AA-HLE for Fable 5 / Sol). Weekly tokens = OpenRouter volume, week ending 2026-07-16 (understates first-party API usage of closed models).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Tool Use tab comparing Kimi K3 vs frontier and open-weights models
- New workbook sheet with MCP Atlas, Toolathlon-Verified, AutomationBench,
  BrowseComp, GDPval-AA Elo, and tau2-bench for Kimi K3, Claude Fable 5,
  GPT-5.6 Sol, Claude Opus 4.8, GLM-5.2, DeepSeek V4 Pro/Flash, MiniMax M3,
  Kimi K2.6, and Nemotron 3 Ultra
- Real-world tool-call leaderboard from OpenRouter's Tool Calls chart
  (raw snapshot committed), plus parallel tool-call API support flags
- CSV export data/csv/tool_use_benchmarks.csv; README documentation

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Top 20 Volume Chart" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By Developer" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Params &amp; Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tool Use" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
@@ -32,7 +33,7 @@
     <numFmt numFmtId="169" formatCode="$0.00"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +60,10 @@
     <font>
       <color rgb="00595959"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -115,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +159,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,6 +493,112 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tool-use benchmarks: MCP Atlas vs Toolathlon-Verified</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tool Use'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tool Use'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tool Use'!$D$6:$D$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Tool Use'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tool Use'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tool Use'!$E$6:$E$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -548,6 +660,33 @@
       <col>0</col>
       <colOff>0</colOff>
       <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3600000"/>
@@ -21239,4 +21378,863 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tool use: Kimi K3 vs closed frontier (Fable 5, GPT-5.6 Sol) and open-weights peers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Agentic tool-calling benchmarks (researched 2026-07-21) plus real-world tool-call traffic on OpenRouter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rows 1-5 (K3, Fable 5, Sol, Opus 4.8, GLM-5.2) share one methodology: Moonshot's Kimi K3 launch table. Remaining rows are vendor-reported under their own harnesses, so compare them loosely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>MCP Atlas (%)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Toolathlon-Verified (%)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>AutomationBench (%)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>BrowseComp (%)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>GDPval-AA (Elo)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>tau2-bench (%)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Parallel tool-call API</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>OpenRouter tool calls, wk of 2026-07-13 (M)</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Weekly tokens (B)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Notes / sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F6" s="32" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>1668</v>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" s="25" t="n">
+        <v>12.051888516</v>
+      </c>
+      <c r="M6" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot launch table (reasoning max, KimiCode/Claude Code harnesses). #1 on AutomationBench-AA (53%) per AA; also leads SpreadsheetBench 2 (34.8) and DeepSearchQA (95.0 F1). BrowseComp hits 90.4 even without context compaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="F7" s="32" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="G7" s="32" t="n">
+        <v>88</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>1760</v>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="25" t="n">
+        <v>375.285408732</v>
+      </c>
+      <c r="M7" s="33" t="inlineStr">
+        <is>
+          <t>Best-in-table on Toolathlon-Verified, GDPval-AA, Job Bench (57.4), OfficeQA Pro (69.9), APEX-Agents (43.3). OpenAI's own table also shows Fable leading Toolathlon (61.7 vs Sol 58.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="F8" s="32" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>1748</v>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="25" t="n">
+        <v>411.249519808</v>
+      </c>
+      <c r="M8" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot table (Codex harness). OpenAI reports SOTA computer use (OSWorld 2.0 62.6%) and Agents' Last Exam 52.7% (+12.2 over Fable); BrowseComp 92.2 in Sol Ultra 4-agent mode. Tau2 from AA leaderboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="F9" s="32" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="G9" s="32" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>1600</v>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="25" t="n">
+        <v>2195.918000173</v>
+      </c>
+      <c r="M9" s="33" t="inlineStr">
+        <is>
+          <t>Closed reference point below the Fable/Sol tier; Moonshot launch table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>1514</v>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" s="32" t="n">
+        <v>43.480658</v>
+      </c>
+      <c r="L10" s="25" t="n">
+        <v>3515.340760024</v>
+      </c>
+      <c r="M10" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot launch table. Z.ai's own blog reports MCP Atlas 77.0 and HLE-with-tools 54.7; built for 'thousands of tool calls' long-horizon sessions. Only row with parallel tool-call API support besides Kimi K2.6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>1554</v>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" s="32" t="n">
+        <v>31.294128</v>
+      </c>
+      <c r="L11" s="25" t="n">
+        <v>2473.441480536</v>
+      </c>
+      <c r="M11" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 technical report, Think-Max mode (Toolathlon standard variant, not Verified).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>69</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>1395</v>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K12" s="32" t="n">
+        <v>70.019233</v>
+      </c>
+      <c r="L12" s="25" t="n">
+        <v>5240.398974088</v>
+      </c>
+      <c r="M12" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 technical report, Think-Max mode. Highest real-world tool-call volume of any paid model on OpenRouter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>1395</v>
+      </c>
+      <c r="I13" s="32" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" s="32" t="n">
+        <v>34.66572</v>
+      </c>
+      <c r="L13" s="25" t="n">
+        <v>3951.536497593</v>
+      </c>
+      <c r="M13" s="33" t="inlineStr">
+        <is>
+          <t>Vendor report / AA-BenchLM mirrors. Native computer use and multimodal input; reported 24-hour autonomous run with ~2,000 tool calls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Kimi K2.6</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>1190</v>
+      </c>
+      <c r="I14" s="32" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="25" t="n">
+        <v>295.80613397</v>
+      </c>
+      <c r="M14" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot K2.7 launch comparison / BenchLM. Best tau2-bench in this set; native agent swarms (300 sub-agents, 4,000 steps); HLE-with-tools 54.0 led all frontier models at release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 Ultra</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="32" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="32" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K15" s="32" t="n">
+        <v>17.958952</v>
+      </c>
+      <c r="L15" s="25" t="n">
+        <v>3316.038765601</v>
+      </c>
+      <c r="M15" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA model card (BF16). Tau2 column shows TauBench V3 average (airline/retail/telecom/banking), a different version from the AA tau2 numbers above. No MCP Atlas or Toolathlon published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>Real-world tool-call traffic on OpenRouter — completed week of 2026-07-13 (total 740M tool calls)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Model (permaslug)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Tool calls (M)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>tencent/hy3-20260706:free</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n">
+        <v>139.987397</v>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>0.1891271908182955</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>xiaomi/mimo-v2.5-20260422</t>
+        </is>
+      </c>
+      <c r="B20" s="25" t="n">
+        <v>109.783504</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>0.148320821407295</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>deepseek/deepseek-v4-flash-20260423</t>
+        </is>
+      </c>
+      <c r="B21" s="25" t="n">
+        <v>70.019233</v>
+      </c>
+      <c r="C21" s="24" t="n">
+        <v>0.09459809328793858</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>z-ai/glm-5.2-20260616</t>
+        </is>
+      </c>
+      <c r="B22" s="25" t="n">
+        <v>43.480658</v>
+      </c>
+      <c r="C22" s="24" t="n">
+        <v>0.05874367892183213</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>minimax/minimax-m3-20260531</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="n">
+        <v>34.66572</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>0.04683443211172505</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>deepseek/deepseek-v4-pro-20260423</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n">
+        <v>31.294128</v>
+      </c>
+      <c r="C24" s="24" t="n">
+        <v>0.04227930974206317</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>google/gemini-2.5-flash</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n">
+        <v>23.553177</v>
+      </c>
+      <c r="C25" s="24" t="n">
+        <v>0.03182105172550704</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>google/gemini-3-flash-preview-20251217</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="n">
+        <v>20.111797</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <v>0.02717164366530669</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>nvidia/nemotron-3-ultra-550b-a55b-20260604:free</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n">
+        <v>17.958952</v>
+      </c>
+      <c r="C27" s="24" t="n">
+        <v>0.02426308521045369</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="n">
+        <v>249.321378</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <v>0.3368406931095831</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Benchmarks: MCP Atlas = multi-step tool use over Model Context Protocol servers (500-task public subset, 100-turn limit, Gemini 3.1 Pro judge). Toolathlon-Verified = multi-tool office/personal workflows; DeepSeek rows use the standard Toolathlon variant. AutomationBench = Zapier-style SaaS automation (600-task subset). BrowseComp = agentic web research. GDPval-AA = Artificial Analysis's Elo for economically valuable professional tasks. tau2-bench = conversational tool use; the Nemotron figure is TauBench V3 (different version).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Kimi K3's launch table is vendor-published: K3 runs at max reasoning effort on Moonshot's preferred harness per benchmark, while competitor numbers mix harnesses and third-party citations. OpenAI's own table shows the same ordering on Toolathlon (Fable 61.7 &gt; Opus 59.9 &gt; Sol 58.0 on the standard variant).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Takeaway: on tool use the three frontier models are within ~1 point on MCP Atlas (Fable 84.7, K3 84.2, Sol 83.6). Fable 5 leads orchestrated professional work (Toolathlon, GDPval-AA, OfficeQA); Sol leads computer use and long-horizon agent runs (OSWorld 62.6, Agents' Last Exam 52.7); K3 leads web research (BrowseComp 91.2) and Zapier-style automation, at roughly half Fable's cost per task ($0.94 vs $2.75 per AA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Real-world traffic tells a different story: OpenRouter's tool-call chart is dominated by cheap open-weights models (Hy3, MiMo-V2.5, DeepSeek V4 Flash, GLM-5.2, MiniMax M3). Fable 5, Sol, and K3 are outside the top 9 tool-callers - premium closed models are used more via first-party APIs and coding products than through OpenRouter tool-calling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Weekly tokens = OpenRouter total volume, week ending 2026-07-16. Kimi K3 launched 2026-07-16, so its volume covers &lt;1 day. Source: OpenRouter (openrouter.ai/rankings), as of 2026-07-21.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add By Cloud Provider tab: open vs closed token volume per serving cloud
- scripts/fetch_endpoint_stats.py snapshots OpenRouter per-endpoint request
  stats for the top 60 model-variant pairs (~96% of weekly volume)
- New workbook sheet distributes weekly tokens across serving providers by
  live request share, rolled up by category (model labs, AI inference
  clouds, US hyperscalers, China hyperscalers) with per-provider table,
  pie chart, and methodology caveats
- CSV export data/csv/cloud_provider_split.csv; raw snapshots committed

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -13,10 +13,12 @@
     <sheet name="By Developer" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Params &amp; Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Tool Use" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="By Cloud Provider" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'By Developer'!$A$1:$F$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'By Cloud Provider'!$A$11:$I$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -66,7 +68,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +93,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,6 +172,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,6 +613,63 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Covered tokens by provider category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'By Cloud Provider'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'By Cloud Provider'!$A$6:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'By Cloud Provider'!$E$6:$E$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -690,6 +761,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -22237,4 +22335,2228 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Where LLM tokens are served: open vs closed volume by cloud / inference provider</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OpenRouter-routed traffic. Weekly volume (week ending 2026-07-16) distributed across each model's serving endpoints by live request share (endpoint snapshot 2026-07-22).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Covers the top 60 model-variant pairs = 56.6T of 59.0T weekly tokens (96%); long-tail models are not attributed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Provider category</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t># providers</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Open-weights tokens (B)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Closed tokens (B)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Total (B)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Share of covered</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Open share within category</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>19554.47309146518</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>5508.585633998697</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>25063.05872546387</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>0.4426598746987205</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>0.7802109593111229</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>17819.76990395207</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>17819.76990395207</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>0.3147300255427007</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>492.8532411557263</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>8096.611272523302</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>8589.46451367903</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0.1517057964473924</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>0.057378808698824</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>4857.684542960011</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>289.246594262</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>5146.931137222011</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>0.09090430331118612</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>0.9438021246932561</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Per provider (estimated weekly tokens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Open-weights tokens (B)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Closed tokens (B)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Total (B)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Share of covered</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Open share</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t># models served</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Novita</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>9724.270864353724</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>9724.270864353724</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>0.1717485710544122</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="19" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Xiaomi</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>8870.93160138263</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>8870.93160138263</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>0.1566770247056617</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>26.44713837728072</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>3643.372603548661</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <v>3669.819741925942</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>0.06481578984122026</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <v>0.007206658701825259</v>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>3538.382602388</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>3538.382602388</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>0.06249436737016682</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>3386.70690058592</v>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>3386.70690058592</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>0.05981549453624832</v>
+      </c>
+      <c r="H16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Minimax</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>2960.380002888598</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>2960.380002888598</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>0.05228577467313941</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Amazon Bedrock</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>66.35561601059729</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>2446.658017106621</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>2513.013633117218</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>0.0443844589017239</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>0.02640479746553853</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>GMICloud</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>2450.343782474326</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>2450.343782474326</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <v>0.04327759367282888</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>StreamLake</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>1976.910329097932</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>1976.910329097932</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <v>0.03491588509426437</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="n">
+        <v>1975.377551852787</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>1975.377551852787</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>0.03488881341914647</v>
+      </c>
+      <c r="H21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>1917.363156021957</v>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="25" t="n">
+        <v>1917.363156021957</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>0.03386417211456755</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>1688.110736887776</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>1688.110736887776</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>0.02981515127318033</v>
+      </c>
+      <c r="H23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>DeepInfra</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>1298.850255655826</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>1298.850255655826</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>0.02294009273644104</v>
+      </c>
+      <c r="H24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="19" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>1193.335205267069</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <v>1193.335205267069</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <v>0.0210765022028378</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="19" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>836.9588164896212</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>289.246594262</v>
+      </c>
+      <c r="F26" s="25" t="n">
+        <v>1126.205410751621</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <v>0.01989086613366289</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <v>0.7431671065503416</v>
+      </c>
+      <c r="I26" s="19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>StepFun</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr"/>
+      <c r="D27" s="25" t="n">
+        <v>891.3895151473678</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="25" t="n">
+        <v>891.3895151473678</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <v>0.01574358402958991</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Google AI Studio</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D28" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>813.2454466009528</v>
+      </c>
+      <c r="F28" s="25" t="n">
+        <v>813.2454466009528</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>0.01436341555254525</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>SiliconFlow</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="n">
+        <v>809.3168766643136</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="25" t="n">
+        <v>809.3168766643136</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>0.01429402975670338</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Poolside</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr"/>
+      <c r="D30" s="25" t="n">
+        <v>658.559920065</v>
+      </c>
+      <c r="E30" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="25" t="n">
+        <v>658.559920065</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>0.01163138365874681</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>AtlasCloud</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>532.3720307492742</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="25" t="n">
+        <v>532.3720307492742</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>0.009402672634890674</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>WandB</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D32" s="25" t="n">
+        <v>467.7431620085956</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="25" t="n">
+        <v>467.7431620085956</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>0.008261207530729116</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="25" t="n">
+        <v>433.7679965249999</v>
+      </c>
+      <c r="F33" s="25" t="n">
+        <v>433.7679965249999</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>0.00766114340206166</v>
+      </c>
+      <c r="H33" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Fireworks</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D34" s="25" t="n">
+        <v>423.1497603469702</v>
+      </c>
+      <c r="E34" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="25" t="n">
+        <v>423.1497603469702</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>0.007473605753621623</v>
+      </c>
+      <c r="H34" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="n">
+        <v>270.604056626115</v>
+      </c>
+      <c r="E35" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="25" t="n">
+        <v>270.604056626115</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>0.004779367080099459</v>
+      </c>
+      <c r="H35" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="19" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Morph</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D36" s="25" t="n">
+        <v>257.5888721012317</v>
+      </c>
+      <c r="E36" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="25" t="n">
+        <v>257.5888721012317</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <v>0.004549494899928883</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="19" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>DigitalOcean</t>
+        </is>
+      </c>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr"/>
+      <c r="D37" s="25" t="n">
+        <v>232.997280134322</v>
+      </c>
+      <c r="E37" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="25" t="n">
+        <v>232.997280134322</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <v>0.004115161998348338</v>
+      </c>
+      <c r="H37" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>Venice</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>224.7711089349958</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="25" t="n">
+        <v>224.7711089349958</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>0.003969872632344325</v>
+      </c>
+      <c r="H38" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" s="19" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Z.AI</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>195.7747477087475</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>195.7747477087475</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>0.003457743375986277</v>
+      </c>
+      <c r="H39" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>184.9627245898924</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="25" t="n">
+        <v>184.9627245898924</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>0.003266783092508609</v>
+      </c>
+      <c r="H40" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>DekaLLM</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>173.4567585682959</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>173.4567585682959</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <v>0.003063566496593562</v>
+      </c>
+      <c r="H41" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B42" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (US)</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>167.0532066335263</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="25" t="n">
+        <v>167.0532066335263</v>
+      </c>
+      <c r="G42" s="24" t="n">
+        <v>0.002950467950716879</v>
+      </c>
+      <c r="H42" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Baidu</t>
+        </is>
+      </c>
+      <c r="B43" s="36" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>126.4522413505007</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="25" t="n">
+        <v>126.4522413505007</v>
+      </c>
+      <c r="G43" s="24" t="n">
+        <v>0.002233379968691311</v>
+      </c>
+      <c r="H43" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="B44" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C44" s="19" t="inlineStr"/>
+      <c r="D44" s="25" t="n">
+        <v>125.6528645351189</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="25" t="n">
+        <v>125.6528645351189</v>
+      </c>
+      <c r="G44" s="24" t="n">
+        <v>0.00221926149876272</v>
+      </c>
+      <c r="H44" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D45" s="25" t="n">
+        <v>121.286905421</v>
+      </c>
+      <c r="E45" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="25" t="n">
+        <v>121.286905421</v>
+      </c>
+      <c r="G45" s="24" t="n">
+        <v>0.002142150602779698</v>
+      </c>
+      <c r="H45" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>Friendli</t>
+        </is>
+      </c>
+      <c r="B46" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>117.9471410623769</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="25" t="n">
+        <v>117.9471410623769</v>
+      </c>
+      <c r="G46" s="24" t="n">
+        <v>0.002083164200173965</v>
+      </c>
+      <c r="H46" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" s="19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Chutes</t>
+        </is>
+      </c>
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>117.0457384175239</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>117.0457384175239</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <v>0.002067243765793053</v>
+      </c>
+      <c r="H47" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>Inceptron</t>
+        </is>
+      </c>
+      <c r="B48" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="n">
+        <v>105.4981014403502</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="25" t="n">
+        <v>105.4981014403502</v>
+      </c>
+      <c r="G48" s="24" t="n">
+        <v>0.00186329118389256</v>
+      </c>
+      <c r="H48" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>NextBit</t>
+        </is>
+      </c>
+      <c r="B49" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="n">
+        <v>96.00186928076782</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="25" t="n">
+        <v>96.00186928076782</v>
+      </c>
+      <c r="G49" s="24" t="n">
+        <v>0.001695570197243796</v>
+      </c>
+      <c r="H49" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>Wafer</t>
+        </is>
+      </c>
+      <c r="B50" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="n">
+        <v>88.49485371775761</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="25" t="n">
+        <v>88.49485371775761</v>
+      </c>
+      <c r="G50" s="24" t="n">
+        <v>0.001562982447085941</v>
+      </c>
+      <c r="H50" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>Decart</t>
+        </is>
+      </c>
+      <c r="B51" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>87.66711499335581</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="25" t="n">
+        <v>87.66711499335581</v>
+      </c>
+      <c r="G51" s="24" t="n">
+        <v>0.001548363053497931</v>
+      </c>
+      <c r="H51" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="B52" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>78.69053643388631</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="25" t="n">
+        <v>78.69053643388631</v>
+      </c>
+      <c r="G52" s="24" t="n">
+        <v>0.001389820108525262</v>
+      </c>
+      <c r="H52" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I52" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>AkashML</t>
+        </is>
+      </c>
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr"/>
+      <c r="D53" s="25" t="n">
+        <v>76.37519382371653</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>76.37519382371653</v>
+      </c>
+      <c r="G53" s="24" t="n">
+        <v>0.001348926884720098</v>
+      </c>
+      <c r="H53" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" s="19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>BaseTen</t>
+        </is>
+      </c>
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C54" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D54" s="25" t="n">
+        <v>73.02369610320724</v>
+      </c>
+      <c r="E54" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="25" t="n">
+        <v>73.02369610320724</v>
+      </c>
+      <c r="G54" s="24" t="n">
+        <v>0.001289733249287788</v>
+      </c>
+      <c r="H54" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>Phala</t>
+        </is>
+      </c>
+      <c r="B55" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>66.10601404721936</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="25" t="n">
+        <v>66.10601404721936</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>0.001167554216566692</v>
+      </c>
+      <c r="H55" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" s="19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>Parasail</t>
+        </is>
+      </c>
+      <c r="B56" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="n">
+        <v>55.75707643627914</v>
+      </c>
+      <c r="E56" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="25" t="n">
+        <v>55.75707643627914</v>
+      </c>
+      <c r="G56" s="24" t="n">
+        <v>0.0009847728778520624</v>
+      </c>
+      <c r="H56" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>Cerebras</t>
+        </is>
+      </c>
+      <c r="B57" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="n">
+        <v>54.93298569387661</v>
+      </c>
+      <c r="E57" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="25" t="n">
+        <v>54.93298569387661</v>
+      </c>
+      <c r="G57" s="24" t="n">
+        <v>0.000970217914359053</v>
+      </c>
+      <c r="H57" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>Io Net</t>
+        </is>
+      </c>
+      <c r="B58" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C58" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D58" s="25" t="n">
+        <v>54.41119710713839</v>
+      </c>
+      <c r="E58" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="25" t="n">
+        <v>54.41119710713839</v>
+      </c>
+      <c r="G58" s="24" t="n">
+        <v>0.0009610021648787194</v>
+      </c>
+      <c r="H58" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>ModelRun</t>
+        </is>
+      </c>
+      <c r="B59" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D59" s="25" t="n">
+        <v>40.13200389271449</v>
+      </c>
+      <c r="E59" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="25" t="n">
+        <v>40.13200389271449</v>
+      </c>
+      <c r="G59" s="24" t="n">
+        <v>0.0007088052583345955</v>
+      </c>
+      <c r="H59" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I59" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>Ionstream</t>
+        </is>
+      </c>
+      <c r="B60" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D60" s="25" t="n">
+        <v>38.08432690530824</v>
+      </c>
+      <c r="E60" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="25" t="n">
+        <v>38.08432690530824</v>
+      </c>
+      <c r="G60" s="24" t="n">
+        <v>0.0006726395034442003</v>
+      </c>
+      <c r="H60" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I60" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>SambaNova</t>
+        </is>
+      </c>
+      <c r="B61" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D61" s="25" t="n">
+        <v>24.26242231379947</v>
+      </c>
+      <c r="E61" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="25" t="n">
+        <v>24.26242231379947</v>
+      </c>
+      <c r="G61" s="24" t="n">
+        <v>0.0004285191579750062</v>
+      </c>
+      <c r="H61" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" s="19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>OpenInference</t>
+        </is>
+      </c>
+      <c r="B62" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D62" s="25" t="n">
+        <v>17.6273925669033</v>
+      </c>
+      <c r="E62" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="25" t="n">
+        <v>17.6273925669033</v>
+      </c>
+      <c r="G62" s="24" t="n">
+        <v>0.0003113322867093969</v>
+      </c>
+      <c r="H62" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I62" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="B63" s="30" t="inlineStr">
+        <is>
+          <t>Model lab</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="n">
+        <v>6.110836075935393</v>
+      </c>
+      <c r="E63" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="25" t="n">
+        <v>6.110836075935393</v>
+      </c>
+      <c r="G63" s="24" t="n">
+        <v>0.0001079286435589644</v>
+      </c>
+      <c r="H63" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B64" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="n">
+        <v>5.977551477588603</v>
+      </c>
+      <c r="E64" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="25" t="n">
+        <v>5.977551477588603</v>
+      </c>
+      <c r="G64" s="24" t="n">
+        <v>0.0001055745915555863</v>
+      </c>
+      <c r="H64" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="19" t="inlineStr">
+        <is>
+          <t>Mancer 2</t>
+        </is>
+      </c>
+      <c r="B65" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr"/>
+      <c r="D65" s="25" t="n">
+        <v>5.547369476965845</v>
+      </c>
+      <c r="E65" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="25" t="n">
+        <v>5.547369476965845</v>
+      </c>
+      <c r="G65" s="24" t="n">
+        <v>9.797678345964769e-05</v>
+      </c>
+      <c r="H65" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I65" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="19" t="inlineStr">
+        <is>
+          <t>Crusoe</t>
+        </is>
+      </c>
+      <c r="B66" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="n">
+        <v>5.498356687317482</v>
+      </c>
+      <c r="E66" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="25" t="n">
+        <v>5.498356687317482</v>
+      </c>
+      <c r="G66" s="24" t="n">
+        <v>9.711112713405578e-05</v>
+      </c>
+      <c r="H66" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I66" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="19" t="inlineStr">
+        <is>
+          <t>Mara</t>
+        </is>
+      </c>
+      <c r="B67" s="35" t="inlineStr">
+        <is>
+          <t>AI inference cloud</t>
+        </is>
+      </c>
+      <c r="C67" s="19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D67" s="25" t="n">
+        <v>3.885253000458657</v>
+      </c>
+      <c r="E67" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="25" t="n">
+        <v>3.885253000458657</v>
+      </c>
+      <c r="G67" s="24" t="n">
+        <v>6.862073880106688e-05</v>
+      </c>
+      <c r="H67" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I67" s="19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
+        <is>
+          <t>Methodology: OpenRouter does not publish per-provider token volume. Each model-variant's weekly tokens are split across its serving endpoints in proportion to each endpoint's live 30-minute request count (openrouter.ai frontend endpoint stats). Requests are a proxy for tokens - providers with atypical request sizes will be over/under-stated - and the 30-minute window is extrapolated to the week, so treat rows as order-of-magnitude estimates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="inlineStr">
+        <is>
+          <t>Categories: 'Model lab' = first-party API of the model's developer (OpenAI, Anthropic, DeepSeek, Moonshot...). 'AI inference cloud' = independent GPU/inference specialists (DeepInfra, Fireworks, Together, Baseten, Novita, Groq...). 'Hyperscaler' = general-purpose public clouds (AWS Bedrock, Azure, Google Vertex/AI Studio, Cloudflare, DigitalOcean; Alibaba, Baidu, Tencent, StreamLake/Kuaishou).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>Closed models can only be served by their lab or licensed hyperscalers, so their provider mix is structurally narrow; open-weights models are served competitively by many independent clouds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="18" t="inlineStr">
+        <is>
+          <t>Google is counted as a hyperscaler (Vertex AI / AI Studio are cloud services) even though it is also the lab behind the Gemini models it serves; the same applies to Alibaba/Tencent/Baidu serving their own models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="inlineStr">
+        <is>
+          <t>Scope caveat: this covers only traffic routed through OpenRouter. Direct first-party API usage (e.g. most OpenAI/Anthropic enterprise traffic) and direct cloud contracts (Bedrock/Vertex/Azure enterprise deals) are not visible here, so hyperscaler and lab shares of the GLOBAL market are far larger than these rows suggest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="inlineStr">
+        <is>
+          <t>Free-tier variant endpoints sometimes expose no live stats (e.g. Tencent Hy3 free promo); those tokens are distributed using the model's standard-variant endpoint mix as a proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
+          <t>Source: OpenRouter (openrouter.ai/rankings), as of 2026-07-22.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A11:I67"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Harnesses & RL Envs tab comparing agent stacks across 8 labs
- New workbook sheet: first-party harnesses, API compatibility, RL
  algorithms/frameworks, disclosed RL environments, and post-training
  openness for Kimi K3, Claude Fable 5, GPT-5.6 Sol, GLM-5/5.2,
  DeepSeek V4, Nemotron 3, MiniMax M3, and Qwen3.7 Max
- Shared-infrastructure reference block (Claude Code, Codex, Kimi Code,
  Terminus-2, Harbor, RepoLaunch, NeMo Gym, slime)
- CSV export data/csv/harness_rl_environments.csv; README documentation

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Params &amp; Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Tool Use" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="By Cloud Provider" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Harnesses &amp; RL Envs" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
@@ -106,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -128,11 +129,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +219,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24559,4 +24612,714 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agent harnesses and RL training environments: Kimi K3 vs open-weights peers and frontier labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>What each lab ships as its agent harness, what is known about its RL post-training stack and environments, and how open that stack is (researched 2026-07-22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Model / family</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>First-party agent harness</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>API / harness compatibility</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>RL algorithm &amp; training stack</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>RL environments (disclosed)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Openness of post-training stack</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Eval harness used</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>Kimi Code CLI (KimiCode harness); Kimi.com / Kimi Work apps; K3 Swarm Max orchestrator for up to 300 parallel sub-agents</t>
+        </is>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI- and Anthropic-compatible APIs; MCP tools. Hard requirement: preserved thinking history - harnesses must pass back all prior reasoning or quality destabilizes; Moonshot recommends verified harnesses (Kimi Code) and warns against mid-session model switches</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
+        <is>
+          <t>Parallel Agent RL (PARL): trainable orchestrator with frozen sub-agents for credit assignment (Agent Swarm lineage from K2.5); per-head Muon optimizer; quantile-balanced MoE routing; trained in preserved-thinking mode; QAT from SFT stage (MXFP4/MXFP8)</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>Not released. Disclosed examples: 24h GPU kernel-optimization sandboxes (H200 + non-NVIDIA GPGPU), 48h chip-design run on open-source EDA tools, internal knowledge-work environments derived from real user-agent workflows. Technical report due with weights (by 2026-07-27)</t>
+        </is>
+      </c>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>Weights open (due 2026-07-27); RL framework and environments not released; contributed KDA prefix-caching to vLLM</t>
+        </is>
+      </c>
+      <c r="I5" s="33" t="inlineStr">
+        <is>
+          <t>KimiCode (own evals); mini-SWE-agent on DeepSWE leaderboard; Claude Code for SWE Marathon/OfficeQA</t>
+        </is>
+      </c>
+      <c r="J5" s="33" t="inlineStr">
+        <is>
+          <t>kimi.com/blog/kimi-k3; Kimi API docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Claude Code (CLI + SDK) - the reference harness most labs benchmark against; Claude Cowork for knowledge work</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic API only (adaptive thinking always on; effort parameter replaces thinking budgets). Harness-level features co-designed with the model: memory tool, context editing / tool-result clearing, compaction, task budgets, code execution, programmatic tool calling; no assistant prefill</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed. Known: RLHF + RL on long-horizon agentic tasks; adaptive reasoning with effort levels (low-&gt;max); Opus 4.8 fallback via safety classifiers (Fable) on cyber/bio/distillation requests</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed. System card documents evaluation (not training) environments across SWE, terminal, multi-agent, computer-use (OSWorld), finance/legal/healthcare agents. Anthropic publishes no RL training data or environments</t>
+        </is>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>Fully closed (weights, data, RL stack); harness (Claude Code) is a product with open plugin/MCP ecosystem</t>
+        </is>
+      </c>
+      <c r="I6" s="33" t="inlineStr">
+        <is>
+          <t>Claude Code / Terminus-2 (AA); vendor system card</t>
+        </is>
+      </c>
+      <c r="J6" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic Fable 5 launch + system card; platform.claude.com docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>Codex suite: Codex CLI (agent loop), Codex Cloud, VS Code extension, App Server (JSON-RPC protocol exposing the harness to products)</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Responses API drives the agent loop (structured context: repo metadata, file tree, diffs, command outputs; automatic compaction; sandboxed execution). Sol defaults to subagent-orchestrator mode; known open issue: subagent config fields hidden, blocking cheap Terra/Luna subagent routing (openai/codex#31814)</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed. Known: RL optimized for multi-step execution (plan-&gt;implement-&gt;validate-&gt;repair) and long uninterrupted runs (~25h reported); reasoning modes incl. 'pro'; models explicitly tuned for the Codex harness</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed. Public signals: Agents' Last Exam-style long-horizon professional workflows (55 fields), OSWorld computer use, terminal tasks. No RL environments or data released</t>
+        </is>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>Fully closed for GPT-5.x; separately ships open-weight gpt-oss models (Apache 2.0, no RL stack)</t>
+        </is>
+      </c>
+      <c r="I7" s="33" t="inlineStr">
+        <is>
+          <t>Codex (own evals and AA Coding Agent Index)</t>
+        </is>
+      </c>
+      <c r="J7" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI 'Unrolling the Codex agent loop', 'Unlocking the Codex harness', GPT-5.6 launch post</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>GLM-5 / GLM-5.2</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>No own CLI - ships Anthropic-native API designed to drop into Claude Code, OpenClaw, Cline etc. (GLM Coding Plan $3-80/mo); positions third-party harnesses as the product surface</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic-native + OpenAI-compatible; parallel tool-call API support (rare among peers); 1M context with dynamic working-memory management for thousands-of-tool-call sessions</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>slime (open-source, Megatron+SGLang) - the disclosed RL framework behind GLM-4.5-&gt;5.2. Sequential pipeline: Reasoning RL -&gt; Agentic RL -&gt; General RL with on-policy cross-stage distillation; fully async decoupled rollout/training; TITO gateway (token-in-token-out); double-sided importance sampling; hybrid rewards (rule-based + ORM + GRM)</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>Most detailed public disclosure of any lab: 10K+ verifiable SWE environments built with RepoLaunch from real issue-PR pairs across 9 languages; synthesized terminal environments in Harbor format (Dockerized, &gt;90% build accuracy); slide-generation environment with executable HTML rendering verification; multi-hop search tasks. Environments themselves not released, but pipeline is documented</t>
+        </is>
+      </c>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>Weights open (MIT); RL framework open (slime on GitHub); environment-building pipelines documented in GLM-5 paper; environment data not released</t>
+        </is>
+      </c>
+      <c r="I8" s="33" t="inlineStr">
+        <is>
+          <t>Claude Code / Terminus-2</t>
+        </is>
+      </c>
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>GLM-5 paper (arXiv:2602.15763); THUDM/slime; z.ai/blog/glm-5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro / Flash</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>No own harness - dual-mode OpenAI + Anthropic-compatible API (drops into Codex- or Claude Code-style harnesses); new XML-based DSML tool-call schema replacing JSON</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI + Anthropic API compatibility; three reasoning modes (non-think / high / max); 1M context</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>Two-stage post-training that replaces mixed RL: (1) domain specialists (math, code, agent, instruction following) each trained with SFT + GRPO where the actor natively functions as its own generative reward model (no separate RM); (2) 10+ specialist teachers merged into one student via multi-teacher on-policy distillation (weighted reverse-KL)</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>Sandbox infrastructure for agentic RL documented in the V4 report (Sec 5.2.5) incl. million-token-context RL rollouts; agentic tool-use data injected already in mid-training. Environments and RL data not released</t>
+        </is>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>Weights open (MIT) incl. base checkpoints; detailed technical report; RL sandbox infra and data not released</t>
+        </is>
+      </c>
+      <c r="I9" s="33" t="inlineStr">
+        <is>
+          <t>Own harness + mini-SWE-agent (DeepSWE); Terminus (TB 2.0)</t>
+        </is>
+      </c>
+      <c r="J9" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Nemotron 3 (Nano/Super/Ultra)</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>NeMo Gym ships out-of-the-box harnesses (incl. Claude Code and Hermes) plus bring-your-own-agent interfaces; served via NVIDIA API / NIM</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible endpoints; models tuned for high-throughput agentic serving on Blackwell (NVFP4)</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>Fully open: NeMo RL + NeMo Gym (RLVR - RL from verifiable rewards). Super trained in 6 disclosed RL stages (RLVR 1-3, SWE 1-2, RLHF) with pass-rate-ordered curriculum; Ultra adds multi-teacher on-policy distillation (MOPD). Also usable with VeRL/Unsloth</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>The only lab that RELEASES its RL environments and data: NeMo Gym environment hub (70+ environments - coding, math, tool use, workplace-assistant agents, SWE-Gym, DAPO-Math, Skywork-OR1...) plus published per-stage RL training blends for Nano/Super/Ultra on Hugging Face with mixing ratios and recipes</t>
+        </is>
+      </c>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>Maximal: open weights + open RL environments + open RL data blends + training recipes + tech reports (NVIDIA Open Model License)</t>
+        </is>
+      </c>
+      <c r="I10" s="33" t="inlineStr">
+        <is>
+          <t>NeMo Evaluator SDK / NeMo Skills; OpenHands for SWE-bench</t>
+        </is>
+      </c>
+      <c r="J10" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA-NeMo/Gym; HF nvidia/Nemotron-RL-*-Training-Blends</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax Agent product; native computer use (only open model here with it); no dedicated CLI - OpenAI/Anthropic-compatible API for third-party harnesses</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI + Anthropic-compatible; text+image+video input; 1M context (MSA sparse attention)</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>CISPO lineage (clips importance-sampling weights instead of token updates - M1 paper); large-scale RL on sandbox-based real-world SWE environments; M1 full RL run cost ~$535K on 512 H800s in 3 weeks. M3-specific recipe not yet published</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>Sandbox-based real-world software engineering environments (disclosed in M1 paper); 24-hour autonomous runs with ~2,000 tool calls reported for M3. Environments not released</t>
+        </is>
+      </c>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>Weights open; CISPO algorithm published; environments and RL data not released</t>
+        </is>
+      </c>
+      <c r="I11" s="33" t="inlineStr">
+        <is>
+          <t>Own agent product; Terminus-2 (AA)</t>
+        </is>
+      </c>
+      <c r="J11" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax-M1 paper (arXiv:2506.13585); M3 launch materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>Qwen Chat + DashScope API; agent-first positioning with native OpenAI- and Anthropic-API compatibility (works in Claude Code / Codex-style harnesses); retains reasoning across turns</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI + Anthropic-compatible; extended-thinking mode (enable_thinking / preserve_thinking); 1M context</t>
+        </is>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed for the closed Max tier. Public signals: QwenWorldBench - internal benchmark using LLMs as world models to simulate agentic environments across 7 domains (Terminal, SWE, MCP, Search, OS, Android, Web) - implies world-model-driven agent training; 35h autonomous kernel-optimization sandbox (Docker + H100, CUTLASS/CUDA docs only) with GPT-5.4 as anti-reward-hacking judge</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>Not released for Max. Open Qwen3.x models ship weights (Apache 2.0) but not RL environments</t>
+        </is>
+      </c>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>Max tier fully closed since late 2025; smaller Qwen models open-weight</t>
+        </is>
+      </c>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>Claude Code harness for agentic evals (per Qwen3.7 blog)</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>Qwen3.7 blog (alibabacloud.com); deeplearning.ai The Batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>Shared harness &amp; RL-environment infrastructure referenced above</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic's CLI harness - de-facto industry reference; GLM, Kimi, and Qwen all advertise compatibility with it and use it in their own evals</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="39" t="n"/>
+      <c r="F16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Codex CLI / App Server</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI's harness; agent loop on the Responses API; also the eval harness for GPT models</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="39" t="n"/>
+      <c r="F17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Kimi Code</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot's CLI; only harness with verified preserved-thinking support for K3</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="n"/>
+      <c r="D18" s="39" t="n"/>
+      <c r="E18" s="39" t="n"/>
+      <c r="F18" s="40" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Terminus-2</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>Terminal-Bench's neutral reference harness, used by Artificial Analysis for cross-model evals</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="39" t="n"/>
+      <c r="E19" s="39" t="n"/>
+      <c r="F19" s="40" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>mini-SWE-agent / OpenHands</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>Open community harnesses used by DeepSWE and SWE-bench leaderboards</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="39" t="n"/>
+      <c r="F20" s="40" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Harbor</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>Dockerized task format for terminal/agent environments; used by Z.ai's synthesized environments and PostTrain Bench</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="n"/>
+      <c r="D21" s="39" t="n"/>
+      <c r="E21" s="39" t="n"/>
+      <c r="F21" s="40" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>RepoLaunch</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>Pipeline that turns real GitHub issue-PR pairs into executable, verifiable SWE environments; basis of Z.ai's 10K+ RL environments</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="39" t="n"/>
+      <c r="F22" s="40" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>NeMo Gym</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA's open RL-environment hub (70+ environments, RLVR datasets, harness integrations incl. Claude Code and Hermes) - the largest open RL environment release</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="n"/>
+      <c r="D23" s="39" t="n"/>
+      <c r="E23" s="39" t="n"/>
+      <c r="F23" s="40" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>slime</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>Z.ai/THUDM's open RL post-training framework (Megatron + SGLang); battle-tested on GLM-4.5 through GLM-5.2; also supports Qwen, DeepSeek, Llama, Kimi K2</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="39" t="n"/>
+      <c r="E24" s="39" t="n"/>
+      <c r="F24" s="40" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Openness spectrum (least to most): OpenAI / Anthropic / Qwen Max disclose harness architecture but no RL environments or data -&gt; Moonshot / DeepSeek / MiniMax release weights + papers but keep environments private -&gt; Z.ai releases weights + the RL framework (slime) and documents its environment pipelines -&gt; NVIDIA releases the entire stack (weights, environments, RL data blends, recipes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>A structural trend across labs: models and harnesses are co-trained and entangled. K3 requires preserved thinking history (unstable in non-verified harnesses), GPT-5.6 Sol is tuned for Codex and Fable 5 for Claude Code, and AA's Coding Agent Index now benchmarks model+harness pairs rather than bare models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>RL environment scale is becoming a disclosed competitive metric: Z.ai reports 10K+ verifiable SWE environments; NVIDIA's NeMo Gym ships 70+ public environments; DeepSeek and Moonshot describe sandbox infrastructure without counts; closed labs disclose nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>Closed-lab rows describe publicly known information only; actual RL stacks are proprietary and may differ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Quantization & KLD tab comparing fidelity profiles across models
- New workbook sheet: release precision/QAT status, external measurability,
  and published KLD at native/4-bit/2-bit tiers for Kimi K3, Kimi K2.6,
  DeepSeek V4 Pro/Flash, GLM-5.2, MiniMax M3, Nemotron 3 Ultra, and the
  unmeasurable closed models (Fable 5, GPT-5.6 Sol, Qwen3.7 Max)
- Measured DeepSeek V4 Flash KLD ladder (Unsloth) as proxy for K3's
  post-weight-release profile; 4-bit format KLD reference table
- Notes on cross-model KLD limits, QAT, and the near-baseline 'silent zone'
- CSV export data/csv/quantization_kld.csv; README documentation

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Tool Use" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="By Cloud Provider" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Harnesses &amp; RL Envs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Quantization &amp; KLD" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
@@ -27,7 +28,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.000"/>
@@ -35,6 +36,7 @@
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="$0.00"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0.0000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -177,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -227,6 +229,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25322,4 +25326,953 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KLD (quantization fidelity): Kimi K3 vs open-weights peers and closed frontier models</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KL divergence measures a quantized variant against ITS OWN full-precision reference; it is not defined across different models (different tokenizers/vocabularies). The comparable question is each model's quantization-fidelity profile. Researched 2026-07-22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Release precision / QAT</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>KLD measurable by outsiders?</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>KLD at native / lossless tier</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>KLD at 4-bit tier</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>KLD at ~2-bit tier</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>Native MXFP4 weights + MXFP8 activations; QAT from the SFT stage (the 4-bit checkpoint IS the model - no higher-precision reference exists)</t>
+        </is>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>Not yet - weights due 2026-07-27; nothing on HF as of 2026-07-22</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
+        <is>
+          <t>~0 by construction (QAT native format)</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>n/a - the native format is already 4-bit</t>
+        </is>
+      </c>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>Pending community quants (Unsloth gates sub-4-bit releases on measured KLD)</t>
+        </is>
+      </c>
+      <c r="I5" s="33" t="inlineStr">
+        <is>
+          <t>Expected to mirror DeepSeek V4 Flash: native MXFP4 experts repack bit-for-bit into GGUF (KLD ~0, 100% top-token agreement). ~1.4TB at MXFP4 vs ~5.6TB BF16-equivalent.</t>
+        </is>
+      </c>
+      <c r="J5" s="33" t="inlineStr">
+        <is>
+          <t>kimi.com/blog/kimi-k3; HF community analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 / K2.7</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Native INT4 QAT for MoE weights, BF16 elsewhere (1T params)</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>Yes (weights public)</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>UD-Q8_K_XL 'truly lossless' (KLD ~0; PPL 1.8419)</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>UD-Q4_K_XL near-lossless: PPL 1.8420 vs 1.8419 lossless (584GB vs 595GB)</t>
+        </is>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>Dynamic 2-bit: PPL 2.4131 (340GB, -43% size); 1/3-bit uploads gated on KLD scores</t>
+        </is>
+      </c>
+      <c r="I6" s="33" t="inlineStr">
+        <is>
+          <t>Because MoE weights are already INT4-native, Q8 repack is bit-exact; only the BF16 non-expert tensors can degrade in smaller quants.</t>
+        </is>
+      </c>
+      <c r="J6" s="33" t="inlineStr">
+        <is>
+          <t>Unsloth Kimi K2.6 guide; unsloth/Kimi-K2.6-GGUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>Native MXFP4 routed experts (96% of params) + FP8/BF16 rest; QAT (284B/13B)</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Yes - the best-measured KLD ladder of any frontier model (see ladder table below)</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>UD-Q8_K_XL: KLD ~0, 100% top-token agreement, all 1,328 tensors bit-identical to official weights</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>UD-Q4_K_XL mean KLD 0.0102 (96.3% top-token); bartowski MXFP4 0.0105; third-party imatrix Q4 0.0290-0.0291 (93.9%)</t>
+        </is>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>0.36-0.42 mean KLD, only ~78% top-token agreement (87-98GB) - the quality cliff</t>
+        </is>
+      </c>
+      <c r="I7" s="33" t="inlineStr">
+        <is>
+          <t>Canonical example of QAT killing the quantization tax at native precision; KLD only reappears in sub-4-bit community compressions.</t>
+        </is>
+      </c>
+      <c r="J7" s="33" t="inlineStr">
+        <is>
+          <t>Unsloth DeepSeek-V4 guide (wikitext-2, ctx 512, 4x B200)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>Same family: native MXFP4 experts + FP8 mixed (1.6T/49B)</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Yes (weights public)</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Native repack lossless by same mechanism as Flash</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>No published ladder (community measured Flash first)</t>
+        </is>
+      </c>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>No published ladder</t>
+        </is>
+      </c>
+      <c r="I8" s="33" t="inlineStr">
+        <is>
+          <t>Expect Flash-like profile; 1.6T scale makes full KLD runs expensive, so trackers prioritized Flash.</t>
+        </is>
+      </c>
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 HF card; Unsloth docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>BF16/FP8 release (753B/40B); no QAT claimed</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>Yes (weights public, MIT)</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>No first-party KLD published</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>Community GGUF quants follow the standard Unsloth Dynamic pattern; no headline KLD table published</t>
+        </is>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="I9" s="33" t="inlineStr">
+        <is>
+          <t>Without QAT, 4-bit quants carry the normal ~0.004-0.012 KLD format tax (see format table below) rather than ~0.</t>
+        </is>
+      </c>
+      <c r="J9" s="33" t="inlineStr">
+        <is>
+          <t>z.ai/blog/glm-5.2; community GGUF repos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>Open weights; MSA sparse-attention architecture</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>Yes (weights public)</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>No KLD published</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="I10" s="33" t="inlineStr">
+        <is>
+          <t>No first-party or major community KLD measurements found as of 2026-07-22.</t>
+        </is>
+      </c>
+      <c r="J10" s="33" t="inlineStr">
+        <is>
+          <t>M3 launch materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 Ultra</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>BF16 reference + NVFP4 post-training-quantized release (550B/55B)</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>Yes, but NVIDIA reports benchmark deltas instead of KLD</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>BF16 = reference (KLD 0 by definition)</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>NVFP4 quality cost measured on benchmarks: AA Intelligence Index 48.2 -&gt; 47.7; GPQA 87.0 -&gt; 87.9; SWE-bench Verified 71.9 -&gt; 69.7; Terminal-Bench 56.4 -&gt; 53.9</t>
+        </is>
+      </c>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="I11" s="33" t="inlineStr">
+        <is>
+          <t>The PTQ (not QAT) counter-example: a real, measurable quality delta between precisions - exactly what QAT-native releases avoid.</t>
+        </is>
+      </c>
+      <c r="J11" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA model card (BF16 vs NVFP4 columns); AA launch article</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed (serving precision unknown)</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>No - no weight access; API exposes no logprobs; no reference distribution exists for outsiders</t>
+        </is>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>Any internal quantization/distillation between training and serving is invisible; users cannot audit serving fidelity.</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic API docs (no logprobs surface)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>No - no weights; API returns top-k logprobs only, and there is no full-precision reference to diverge from</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="H13" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="I13" s="33" t="inlineStr">
+        <is>
+          <t>Top-k logprobs allow drift monitoring over time, but not KLD against a reference checkpoint.</t>
+        </is>
+      </c>
+      <c r="J13" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI API docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed (API-only tier)</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>No - closed weights since late 2025 for the Max tier</t>
+        </is>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>Unmeasurable</t>
+        </is>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba's open Qwen3.x models are measurable (community GGUF KLD tables exist, e.g. Qwen3.6-27B used as the format reference below); the Max tier is not.</t>
+        </is>
+      </c>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>Qwen release notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Measured KLD ladder - DeepSeek V4 Flash (closest public proxy for K3's future ladder; Unsloth, wikitext-2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Quant</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Size (GB)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Mean KLD</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>RMS delta-p (%)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Same top token (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Official checkpoint (reference)</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>156.4</v>
+      </c>
+      <c r="C18" s="41" t="n">
+        <v>4.5319</v>
+      </c>
+      <c r="D18" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="42" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Unsloth UD-Q8_K_XL</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="C19" s="41" t="n">
+        <v>4.5319</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Unsloth UD-Q4_K_XL</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>155.1</v>
+      </c>
+      <c r="C20" s="41" t="n">
+        <v>4.5335</v>
+      </c>
+      <c r="D20" s="41" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>96.28</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>bartowski MXFP4</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>156</v>
+      </c>
+      <c r="C21" s="41" t="n">
+        <v>4.5351</v>
+      </c>
+      <c r="D21" s="41" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="E21" s="42" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>96.18000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>antirez Q4KExperts-F16 (imatrix)</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>164.6</v>
+      </c>
+      <c r="C22" s="41" t="n">
+        <v>4.5743</v>
+      </c>
+      <c r="D22" s="41" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="E22" s="42" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="F22" s="42" t="n">
+        <v>93.95</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>antirez mixed L37-42-Q4K (imatrix)</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="C23" s="41" t="n">
+        <v>5.8169</v>
+      </c>
+      <c r="D23" s="41" t="n">
+        <v>0.3605</v>
+      </c>
+      <c r="E23" s="42" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <v>79.73999999999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>antirez IQ2XXS (imatrix)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="C24" s="41" t="n">
+        <v>6.0808</v>
+      </c>
+      <c r="D24" s="41" t="n">
+        <v>0.4079</v>
+      </c>
+      <c r="E24" s="42" t="n">
+        <v>22.23</v>
+      </c>
+      <c r="F24" s="42" t="n">
+        <v>78.15000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>4-bit-class format KLD vs FP16 (measured on Qwen3.6-27B; lower = closer to full precision; MXFP4 is K3's native format)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Bits per weight</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Q4_K_M (classic GGUF)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>oQ ('optimal Q')</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>MXFP4/MXFP6</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>UD-MLX</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="41" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="C28" s="41" t="n">
+        <v>0.0078</v>
+      </c>
+      <c r="D28" s="41" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="E28" s="41" t="n">
+        <v>0.0042</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="B29" s="41" t="n">
+        <v>0.0094</v>
+      </c>
+      <c r="C29" s="41" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="D29" s="41" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="E29" s="41" t="n">
+        <v>0.0031</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" s="41" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="C30" s="41" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="D30" s="41" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="E30" s="41" t="n">
+        <v>0.0017</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" s="41" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="C31" s="41" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="D31" s="41" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Why there is no 'K3 KLD vs Fable 5 KLD' number: KL divergence compares two probability distributions over the same vocabulary. Different models have different tokenizers and no shared reference, so cross-model KLD is undefined. The comparable dimension is how faithfully each model's served/compressed form reproduces its own reference - and whether outsiders can measure that at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>The open-weights frontier has engineered the quantization tax away: K3, K2.x, and DeepSeek V4 are quantization-aware-trained so the low-precision checkpoint IS the model (KLD ~0 at native precision). KLD only becomes a live issue for sub-4-bit community compressions, where ~2-bit costs 0.36+ KLD and ~22% top-token disagreement (the quality cliff).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>Closed models are unauditable on this axis: Anthropic exposes no logprobs, OpenAI only top-k, and neither releases a reference checkpoint - so serving fidelity is a trust relationship, not a measurement. With open models you can verify token-level fidelity yourself (Unsloth verified DeepSeek V4 Flash bit-identical).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>Interpretation caveat (July 2026 community finding): KLD has a 'silent zone' near baseline where further KLD reductions do not translate into quality gains; Unsloth and the 'Accuracy is Not All You Need' paper recommend pairing KLD with flip-sensitive benchmarks (e.g. Aider) rather than reading tiny KLD deltas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>Kimi K3 status: weights promised by 2026-07-27 (not on Hugging Face as of 2026-07-22). Expect an Unsloth-style measured ladder within days of release; until then the K3 row is by-construction reasoning, not measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Nemotron 3 Ultra is the post-training-quantization counter-example: NVIDIA ships BF16 + NVFP4 and reports the quality delta on benchmarks (AA Index 48.2 vs 47.7) rather than KLD.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Training Data tab and compile CSV tables into data-only workbook
- New 'Training Data' sheet: vendor-disclosed pretraining corpus sizes for
  15 model families (MiMo-V2.5 48T, Llama 4 Scout 40T, DeepSeek V4 32T,
  GLM-5 27T, Nemotron 3 25T, Kimi K2 15.5T; closed labs undisclosed) with
  tokens-per-param ratios, pipeline notes, and disclosed-corpus chart
- data/llm_data_tables.xlsx: every CSV table compiled into one data-only
  Excel workbook (auto-generated by the build script)
- CSV export data/csv/training_data.csv; README documentation

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/llm_pricing_vs_token_volume.xlsx
+++ b/data/llm_pricing_vs_token_volume.xlsx
@@ -16,6 +16,7 @@
     <sheet name="By Cloud Provider" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Harnesses &amp; RL Envs" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Quantization &amp; KLD" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Training Data" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Model Comparison'!$A$1:$P$305</definedName>
@@ -28,7 +29,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.000"/>
@@ -37,6 +38,7 @@
     <numFmt numFmtId="169" formatCode="$0.00"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
     <numFmt numFmtId="171" formatCode="0.0000"/>
+    <numFmt numFmtId="172" formatCode="#,##0x"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -179,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -231,6 +233,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -727,6 +738,85 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Disclosed pretraining corpus size (T tokens)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Training Data'!B28</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Training Data'!$A$29:$A$36</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Training Data'!$B$29:$B$36</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -845,6 +935,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1367,6 +1484,877 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pretraining dataset sizes: what each lab disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Vendor-disclosed pretraining corpus sizes (trillions of tokens) for the models featured in this workbook; researched 2026-07-24. Closed labs disclose nothing, so their rows document that asymmetry rather than a number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Total params (B)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Pretraining tokens (T)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Tokens per total param</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Disclosure status</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Data composition / pipeline notes</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="68" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D5" s="43" t="n">
+        <v>2800</v>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed (tech report due with weights, 2026-07-27)</t>
+        </is>
+      </c>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>Pipeline disclosed without quantities: web+code+vision pretraining, long-context mid-training toward 1M, SFT, RLVR. Predecessor Kimi K2 (1T params) disclosed 15.5T tokens, so K3's corpus is presumably well beyond that; treat any specific figure circulating now as an estimate.</t>
+        </is>
+      </c>
+      <c r="I5" s="33" t="inlineStr">
+        <is>
+          <t>kimi.com/blog/kimi-k3; Kimi K2 paper (arXiv:2507.20534)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="68" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K2 / K2.6</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E6" s="44" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="F6" s="45" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed for K2 base (K2.6/K2.7 increments not broken out)</t>
+        </is>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>15.5T curated tokens across web text, code, mathematics, knowledge; MuonClip optimizer, 4,096-token pretraining window.</t>
+        </is>
+      </c>
+      <c r="I6" s="33" t="inlineStr">
+        <is>
+          <t>Kimi K2 paper (arXiv:2507.20534)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>Anthropic discloses neither corpus size nor parameter count for any frontier model.</t>
+        </is>
+      </c>
+      <c r="I7" s="33" t="inlineStr">
+        <is>
+          <t>Fable 5 system card (no training-data quantities)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="68" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>OpenAI stopped disclosing training-data scale after GPT-3 (300B tokens, 2020). gpt-oss open-weight models also ship without a precise token count ('trillions of tokens').</t>
+        </is>
+      </c>
+      <c r="I8" s="33" t="inlineStr">
+        <is>
+          <t>GPT-5.6 launch materials (no training-data quantities)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Gemini 3.x</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>No corpus quantities disclosed for the Gemini series.</t>
+        </is>
+      </c>
+      <c r="I9" s="33" t="inlineStr">
+        <is>
+          <t>Gemini model cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>GLM-5 / 5.1 / 5.2</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>Z.ai (Zhipu)</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="n">
+        <v>753</v>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" s="45" t="n">
+        <v>35.85657370517928</v>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed (GLM-5 base, which 5.1/5.2 build on)</t>
+        </is>
+      </c>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>27T-token corpus prioritizing code and reasoning early; distinct mid-training phase extends context 4K-&gt;200K with long-context agentic data.</t>
+        </is>
+      </c>
+      <c r="I10" s="33" t="inlineStr">
+        <is>
+          <t>GLM-5 paper (arXiv:2602.15763)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="68" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E11" s="44" t="n">
+        <v>32</v>
+      </c>
+      <c r="F11" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed ('more than 32T tokens', shared corpus with Flash)</t>
+        </is>
+      </c>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>Agentic tool-use data injected already in mid-training; FP8-mixed pretraining with MXFP4 on expert weights.</t>
+        </is>
+      </c>
+      <c r="I11" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="n">
+        <v>284</v>
+      </c>
+      <c r="E12" s="44" t="n">
+        <v>32</v>
+      </c>
+      <c r="F12" s="45" t="n">
+        <v>112.6760563380282</v>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed ('more than 32T tokens', shared corpus with Pro)</t>
+        </is>
+      </c>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>Same &gt;32T corpus as V4 Pro; the small variant is heavily over-trained relative to its size (~113 tokens per param).</t>
+        </is>
+      </c>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4 report (arXiv:2606.19348)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Qwen3.7 Max</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba (Qwen)</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed (closed tier)</t>
+        </is>
+      </c>
+      <c r="H13" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba disclosed 36T tokens for the open Qwen3 generation (2025) but publishes no quantities for the closed Max tier.</t>
+        </is>
+      </c>
+      <c r="I13" s="33" t="inlineStr">
+        <is>
+          <t>Qwen3 technical report (2025); Qwen3.7 launch blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="68" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Nemotron 3 (Nano/Super/Ultra)</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E14" s="44" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed AND largely released - the only lab that ships much of the corpus itself</t>
+        </is>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>25T tokens in two phases (23.5T diverse + 1.5T high-quality) + 121B long-context phase; 16 data categories. ~8-10T tokens (~40-50% of the blend) released as open datasets (Nemotron-CC-v2.x, CC-Math, Pretraining-Code, Specialized). Documented for Nano/Super; Ultra follows the same data program.</t>
+        </is>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>NVIDIA Nemotron 3 pretraining docs + Nano tech report; HF Nemotron pretraining dataset collections</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>MiMo-V2.5</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>Xiaomi</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>310</v>
+      </c>
+      <c r="E15" s="44" t="n">
+        <v>48</v>
+      </c>
+      <c r="F15" s="45" t="n">
+        <v>154.8387096774194</v>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed - largest disclosed corpus of any model here</t>
+        </is>
+      </c>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>~48T tokens, FP8 mixed precision, five-stage pipeline (text pretraining, projector warmup, multimodal pretraining, SFT/agentic post-training with 32K-&gt;256K-&gt;1M context extension, RL+MOPD). ~155 tokens per param - the most over-trained large model on this list.</t>
+        </is>
+      </c>
+      <c r="I15" s="33" t="inlineStr">
+        <is>
+          <t>XiaomiMiMo/MiMo-V2.5 HF card; mimo.xiaomi.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="68" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Hy3</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>295</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H16" s="33" t="inlineStr">
+        <is>
+          <t>295B/21B MoE (192 experts, top-8 routing); Tencent's model card discusses post-training scale-up but no corpus count.</t>
+        </is>
+      </c>
+      <c r="I16" s="33" t="inlineStr">
+        <is>
+          <t>Tencent Hy3 model card; SiliconFlow explainer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="68" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax M3</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>Undisclosed</t>
+        </is>
+      </c>
+      <c r="H17" s="33" t="inlineStr">
+        <is>
+          <t>No corpus size published for M3; total params also not officially stated (third-party estimates ~200-400B).</t>
+        </is>
+      </c>
+      <c r="I17" s="33" t="inlineStr">
+        <is>
+          <t>M3 launch materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="68" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>Llama 4 Scout</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>109</v>
+      </c>
+      <c r="E18" s="44" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" s="45" t="n">
+        <v>366.9724770642202</v>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed (2025)</t>
+        </is>
+      </c>
+      <c r="H18" s="33" t="inlineStr">
+        <is>
+          <t>~40T multimodal tokens - highest tokens-per-param ratio here (~367x); 10M-token context via iRoPE.</t>
+        </is>
+      </c>
+      <c r="I18" s="33" t="inlineStr">
+        <is>
+          <t>Meta Llama 4 launch blog (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="68" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>Llama 4 Maverick</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>Open-weights</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>400</v>
+      </c>
+      <c r="E19" s="44" t="n">
+        <v>22</v>
+      </c>
+      <c r="F19" s="45" t="n">
+        <v>55</v>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>Disclosed (2025)</t>
+        </is>
+      </c>
+      <c r="H19" s="33" t="inlineStr">
+        <is>
+          <t>~22T multimodal tokens.</t>
+        </is>
+      </c>
+      <c r="I19" s="33" t="inlineStr">
+        <is>
+          <t>Meta Llama 4 launch blog (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Disclosure asymmetry mirrors the rest of this workbook: every disclosed corpus size belongs to an open-weights model; Anthropic, OpenAI, Google, and Alibaba's closed tier publish nothing. NVIDIA goes furthest, releasing ~8-10T tokens of the actual corpus as open datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Tokens-per-parameter is a rough over-training indicator (Chinchilla-optimal is ~20x): DeepSeek V4 Pro sits near 20x while small-model releases (MiMo-V2.5 ~155x, Llama 4 Scout ~367x, Nemotron 3 Super ~208x) are heavily over-trained to maximize quality per active parameter at inference time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>Counts are vendor-reported and not independently verifiable; token counts also are not comparable apples-to-apples across labs (different tokenizers, dedup policies, and multimodal counting).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Kimi K3's corpus size should be published with its technical report alongside the weights (due 2026-07-27); this row can then be updated from 'undisclosed' to a disclosed figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Pretraining corpus size is distinct from post-training/RL data, which is covered in the Harnesses &amp; RL Envs tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Pretraining tokens (T)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Kimi K2 / K2.6</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GLM-5 / 5.1 / 5.2</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nemotron 3 (Nano/Super/Ultra)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MiMo-V2.5</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Llama 4 Scout</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Llama 4 Maverick</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>